<commit_message>
Add menu plan workbook
</commit_message>
<xml_diff>
--- a/data/減脂追蹤.xlsx
+++ b/data/減脂追蹤.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日紀錄" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="菜單規劃" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'每日紀錄'!$A$4:$P$4</definedName>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +56,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -102,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -130,6 +136,18 @@
     <xf numFmtId="166" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -993,4 +1011,998 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>減脂菜單規劃｜一週四練</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>保留原始菜單作為參考；日常只需在「每日紀錄」填入 Calories、Protein、Carbs、Fat。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>訓練日菜單｜晚上重訓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>時間</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>餐次</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>雞胸（生重）</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>白飯（熟重）</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>生米約米杯</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>其他食物</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>青菜</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>早餐</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>120 g</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>約 1/3 杯</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>全蛋 2 顆</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>正常吃，不需刻意低碳</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>午餐</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>150 g（半盒）</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>180 g</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>約 0.55 杯</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>鯖魚日加台糖水煮鯖魚 1/2 罐</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>200 g</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>鯖魚每週 3 次即可</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>訓前餐</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>180 g</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>約 0.55 杯</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>乳清 1 scoop＋香蕉 1 根</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>盡量距訓練 1.5–2.5 小時</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>19:30–21:00</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>重訓</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>水</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>依實際訓練時間前後平移</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>訓後晚餐</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>150 g（半盒）</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>160 g</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>約 1/2 杯</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>全蛋 2 顆</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>200 g</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>晚間吃白飯沒有問題</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>睡前</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>視需要補蛋白</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>乳清 0.5–1 scoop</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>當天蛋白質足夠可省略</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>每日合計</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n"/>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>300 g（1盒）</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>640 g</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>約 1.9–2.0 杯</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>全蛋 4 顆＋乳清 1.5–2 scoop＋香蕉 1 根</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>至少 400 g</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>休息日菜單</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>時間</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>餐次</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>雞胸（生重）</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>白飯（熟重）</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>生米約米杯</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>其他食物</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>青菜</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>早餐</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>100 g</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>約 0.30 杯</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>全蛋 2 顆＋乳清 1 scoop</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>休息日仍保留碳水</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>午餐</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>150 g（半盒）</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>200 g</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>約 0.60 杯</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>鯖魚日加台糖水煮鯖魚 1/2 罐</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>300 g</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>鯖魚每週 3 次即可</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>晚餐</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>150 g（半盒）</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>150 g</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>約 0.45 杯</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>全蛋 2 顆</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>300 g</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>睡前</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>乳清 0.5–1 scoop</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>依當天蛋白質攝取調整</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>每日合計</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>300 g（1盒）</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>450 g</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>約 1.35–1.4 杯</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>全蛋 4 顆＋乳清 1.5–2 scoop</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>約 600 g</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>每週安排</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>星期</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>類型</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>雞胸</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>生米</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>鯖魚</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>蛋</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>週一</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>訓練日</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>1盒</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>約2杯</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>1/2罐</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>4顆</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>週二</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>訓練日</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>1盒</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>約2杯</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>4顆</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>週三</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>休息日</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>1盒</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>約1.4杯</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>4顆</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>週四</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>訓練日</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>1盒</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>約2杯</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>1/2罐</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>4顆</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>週五</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>休息日</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>1盒</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>約1.4杯</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>4顆</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>週六</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>訓練日</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>1盒</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>約2杯</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>1/2罐</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>4顆</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>週日</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>休息日</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>1盒</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>約1.4杯</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>4顆</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>每週採買建議</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>數量</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>雞胸 300 g/盒</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>7 盒</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>台糖水煮鯖魚</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>2 罐即可（實吃 1.5 罐）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>雞蛋</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>28 顆</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>生米</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>約 12.2 米杯/週</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>香蕉</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>至少 4 根</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>青菜</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>約 3.4 kg/週以上</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>乳清</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>約 11–14 scoop/週</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A35:B35"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update rest day and replacement menus
</commit_message>
<xml_diff>
--- a/data/減脂追蹤.xlsx
+++ b/data/減脂追蹤.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -148,6 +148,24 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1019,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1096,27 +1114,27 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>早餐</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>120 g</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>約 1/3 杯</t>
         </is>
@@ -1126,7 +1144,7 @@
           <t>全蛋 2 顆</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1138,27 +1156,27 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>午餐</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>150 g（半盒）</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>180 g</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>約 0.55 杯</t>
         </is>
@@ -1168,7 +1186,7 @@
           <t>鯖魚日加台糖水煮鯖魚 1/2 罐</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr">
+      <c r="G7" s="21" t="inlineStr">
         <is>
           <t>200 g</t>
         </is>
@@ -1180,27 +1198,27 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>訓前餐</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>180 g</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>約 0.55 杯</t>
         </is>
@@ -1210,7 +1228,7 @@
           <t>乳清 1 scoop＋香蕉 1 根</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1222,27 +1240,27 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>19:30–21:00</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>重訓</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1252,7 +1270,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1264,27 +1282,27 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>訓後晚餐</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>150 g（半盒）</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>160 g</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>約 1/2 杯</t>
         </is>
@@ -1294,7 +1312,7 @@
           <t>全蛋 2 顆</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>200 g</t>
         </is>
@@ -1306,27 +1324,27 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>睡前</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>視需要補蛋白</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1336,7 +1354,7 @@
           <t>乳清 0.5–1 scoop</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1348,23 +1366,23 @@
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>每日合計</t>
         </is>
       </c>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="B12" s="22" t="n"/>
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>300 g（1盒）</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>640 g</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>約 1.9–2.0 杯</t>
         </is>
@@ -1374,12 +1392,12 @@
           <t>全蛋 4 顆＋乳清 1.5–2 scoop＋香蕉 1 根</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>至少 400 g</t>
         </is>
       </c>
-      <c r="H12" s="16" t="n"/>
+      <c r="H12" s="22" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -1431,202 +1449,160 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>07:30</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>早餐</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>午餐</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>150 g（半盒）</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>200 g</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>約 0.60 杯</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>鯖魚日加台糖水煮鯖魚 1/2 罐</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="inlineStr">
+        <is>
+          <t>300 g</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>鯖魚每週 3 次即可</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>下午茶</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>100 g</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>約 0.30 杯</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
-        <is>
-          <t>全蛋 2 顆＋乳清 1 scoop</t>
-        </is>
-      </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>全蛋 2 顆＋乳清 1–1.5 scoop</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H17" s="15" t="inlineStr">
-        <is>
-          <t>休息日仍保留碳水</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>午餐</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>把原早餐內容移到下午茶；若蛋白質不足再補 0.5 scoop</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>晚餐</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>150 g（半盒）</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>200 g</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>約 0.60 杯</t>
-        </is>
-      </c>
-      <c r="F18" s="15" t="inlineStr">
-        <is>
-          <t>鯖魚日加台糖水煮鯖魚 1/2 罐</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>150 g</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>約 0.45 杯</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>全蛋 2 顆</t>
+        </is>
+      </c>
+      <c r="G19" s="21" t="inlineStr">
         <is>
           <t>300 g</t>
         </is>
       </c>
-      <c r="H18" s="15" t="inlineStr">
-        <is>
-          <t>鯖魚每週 3 次即可</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>晚餐</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>150 g（半盒）</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>150 g</t>
-        </is>
-      </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>約 0.45 杯</t>
-        </is>
-      </c>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>全蛋 2 顆</t>
-        </is>
-      </c>
-      <c r="G19" s="14" t="inlineStr">
-        <is>
-          <t>300 g</t>
-        </is>
-      </c>
       <c r="H19" s="15" t="inlineStr"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>睡前</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>乳清 0.5–1 scoop</t>
-        </is>
-      </c>
-      <c r="G20" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>依當天蛋白質攝取調整</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>每日合計</t>
         </is>
       </c>
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr"/>
+      <c r="C20" s="22" t="inlineStr">
         <is>
           <t>300 g（1盒）</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
         <is>
           <t>450 g</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>約 1.35–1.4 杯</t>
         </is>
       </c>
-      <c r="F21" s="17" t="inlineStr">
-        <is>
-          <t>全蛋 4 顆＋乳清 1.5–2 scoop</t>
-        </is>
-      </c>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>全蛋 4 顆＋乳清 1–1.5 scoop</t>
+        </is>
+      </c>
+      <c r="G20" s="22" t="inlineStr">
         <is>
           <t>約 600 g</t>
         </is>
       </c>
-      <c r="H21" s="16" t="n"/>
+      <c r="H20" s="22" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
@@ -1668,27 +1644,27 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>週一</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>訓練日</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="C26" s="21" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>約2杯</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>1/2罐</t>
         </is>
@@ -1700,27 +1676,27 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>週二</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>訓練日</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="21" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>約2杯</t>
         </is>
       </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1732,27 +1708,27 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>週三</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>休息日</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>約1.4杯</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1764,27 +1740,27 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>週四</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>訓練日</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>約2杯</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>1/2罐</t>
         </is>
@@ -1796,27 +1772,27 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>週五</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>休息日</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t>約1.4杯</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1828,27 +1804,27 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>週六</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>訓練日</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="21" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D31" s="14" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>約2杯</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>1/2罐</t>
         </is>
@@ -1860,27 +1836,27 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>週日</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B32" s="21" t="inlineStr">
         <is>
           <t>休息日</t>
         </is>
       </c>
-      <c r="C32" s="14" t="inlineStr">
+      <c r="C32" s="21" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D32" s="14" t="inlineStr">
+      <c r="D32" s="21" t="inlineStr">
         <is>
           <t>約1.4杯</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
+      <c r="E32" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1911,97 +1887,273 @@
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>雞胸 300 g/盒</t>
         </is>
       </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="21" t="inlineStr">
         <is>
           <t>7 盒</t>
         </is>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>台糖水煮鯖魚</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>2 罐即可（實吃 1.5 罐）</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="A39" s="21" t="inlineStr">
         <is>
           <t>雞蛋</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="21" t="inlineStr">
         <is>
           <t>28 顆</t>
         </is>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="A40" s="21" t="inlineStr">
         <is>
           <t>生米</t>
         </is>
       </c>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="B40" s="21" t="inlineStr">
         <is>
           <t>約 12.2 米杯/週</t>
         </is>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="A41" s="21" t="inlineStr">
         <is>
           <t>香蕉</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>至少 4 根</t>
         </is>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="14" t="inlineStr">
+      <c r="A42" s="21" t="inlineStr">
         <is>
           <t>青菜</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B42" s="21" t="inlineStr">
         <is>
           <t>約 3.4 kg/週以上</t>
         </is>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="A43" s="21" t="inlineStr">
         <is>
           <t>乳清</t>
         </is>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="21" t="inlineStr">
         <is>
           <t>約 11–14 scoop/週</t>
         </is>
       </c>
     </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>替換方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>替換食物</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>可替代</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>建議份量</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>使用方式</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>蛋白質</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>碳水</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>脂肪</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="48" customHeight="1">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>711 鮪魚飯糰</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>白飯＋部分蛋白質</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>1 顆</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>可放午餐或下午茶；蛋白質不足時再補乳清或無糖豆漿</t>
+        </is>
+      </c>
+      <c r="E48" s="23" t="inlineStr">
+        <is>
+          <t>依包裝</t>
+        </is>
+      </c>
+      <c r="F48" s="15" t="inlineStr">
+        <is>
+          <t>依包裝</t>
+        </is>
+      </c>
+      <c r="G48" s="23" t="inlineStr">
+        <is>
+          <t>依包裝</t>
+        </is>
+      </c>
+      <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>不同口味與大小以包裝標示為準</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="48" customHeight="1">
+      <c r="A49" s="23" t="inlineStr">
+        <is>
+          <t>雞胗</t>
+        </is>
+      </c>
+      <c r="B49" s="23" t="inlineStr">
+        <is>
+          <t>雞胸</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>150–200 g</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>選清滷或少油版本，替代一份雞胸；當天脂肪偏高時減少額外油脂</t>
+        </is>
+      </c>
+      <c r="E49" s="23" t="inlineStr">
+        <is>
+          <t>依份量</t>
+        </is>
+      </c>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="23" t="inlineStr">
+        <is>
+          <t>依烹調</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>注意滷汁、麻油與其他調味</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="48" customHeight="1">
+      <c r="A50" s="23" t="inlineStr">
+        <is>
+          <t>地瓜</t>
+        </is>
+      </c>
+      <c r="B50" s="23" t="inlineStr">
+        <is>
+          <t>白飯</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>150–200 g</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>可放午餐或下午茶，依當日 Carbs 差額調整份量</t>
+        </is>
+      </c>
+      <c r="E50" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>依份量</t>
+        </is>
+      </c>
+      <c r="G50" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="15" t="inlineStr">
+        <is>
+          <t>以熟重估算，實際仍以紀錄值為準</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A46:H46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add today food log
</commit_message>
<xml_diff>
--- a/data/減脂追蹤.xlsx
+++ b/data/減脂追蹤.xlsx
@@ -253,7 +253,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyRecordTable" displayName="DailyRecordTable" ref="A4:P4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyRecordTable" displayName="DailyRecordTable" ref="A4:P5" headerRowCount="1">
   <autoFilter ref="A4:P4"/>
   <tableColumns count="16">
     <tableColumn id="1" name="日期"/>
@@ -699,21 +699,62 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="6" t="n"/>
-      <c r="M5" s="7" t="n"/>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="8" t="n"/>
+      <c r="A5" s="4" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>365</v>
+      </c>
+      <c r="D5" s="7">
+        <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$12,IF($B5="REST",'設定'!$D$12,"")))</f>
+        <v/>
+      </c>
+      <c r="E5" s="7">
+        <f>IF(OR($C5="",$D5=""),"",$D5-$C5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="G5" s="7">
+        <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$13,IF($B5="REST",'設定'!$D$13,"")))</f>
+        <v/>
+      </c>
+      <c r="H5" s="7">
+        <f>IF(OR($F5="",$G5=""),"",$G5-$F5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="J5" s="7">
+        <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$14,IF($B5="REST",'設定'!$D$14,"")))</f>
+        <v/>
+      </c>
+      <c r="K5" s="7">
+        <f>IF(OR($I5="",$J5=""),"",$J5-$I5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="M5" s="7">
+        <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$15,IF($B5="REST",'設定'!$D$15,"")))</f>
+        <v/>
+      </c>
+      <c r="N5" s="7">
+        <f>IF(OR($L5="",$M5=""),"",$M5-$L5)</f>
+        <v/>
+      </c>
+      <c r="O5" s="8">
+        <f>IF($A5="","",IF($B5="","請先填 Day_Type（TRAINING 或 REST）",IF(OR($C5="",$F5="",$I5="",$L5=""),"請補齊 Calories、Protein、Carbs、Fat",IF($H5&gt;0,"優先補蛋白質。",IF($K5&gt;0,"蛋白質已足夠，優先補碳水，例如白飯或香蕉。",IF($N5&gt;0,"優先補脂肪。",IF($E5&gt;0,"三大營養素已達最低，熱量尚差；可補少量主食。","已達每日最低目標；蛋白質足夠，不需補充乳清。")))))))</f>
+        <v/>
+      </c>
       <c r="P5" s="9" t="n"/>
     </row>
   </sheetData>
@@ -1114,27 +1155,27 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>早餐</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D6" s="21" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>120 g</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="E6" s="23" t="inlineStr">
         <is>
           <t>約 1/3 杯</t>
         </is>
@@ -1144,7 +1185,7 @@
           <t>全蛋 2 顆</t>
         </is>
       </c>
-      <c r="G6" s="21" t="inlineStr">
+      <c r="G6" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1156,27 +1197,27 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>午餐</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>150 g（半盒）</t>
         </is>
       </c>
-      <c r="D7" s="21" t="inlineStr">
+      <c r="D7" s="23" t="inlineStr">
         <is>
           <t>180 g</t>
         </is>
       </c>
-      <c r="E7" s="21" t="inlineStr">
+      <c r="E7" s="23" t="inlineStr">
         <is>
           <t>約 0.55 杯</t>
         </is>
@@ -1186,7 +1227,7 @@
           <t>鯖魚日加台糖水煮鯖魚 1/2 罐</t>
         </is>
       </c>
-      <c r="G7" s="21" t="inlineStr">
+      <c r="G7" s="23" t="inlineStr">
         <is>
           <t>200 g</t>
         </is>
@@ -1198,27 +1239,27 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>訓前餐</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>180 g</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="E8" s="23" t="inlineStr">
         <is>
           <t>約 0.55 杯</t>
         </is>
@@ -1228,7 +1269,7 @@
           <t>乳清 1 scoop＋香蕉 1 根</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
+      <c r="G8" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1240,27 +1281,27 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>19:30–21:00</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>重訓</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="21" t="inlineStr">
+      <c r="E9" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1270,7 +1311,7 @@
           <t>水</t>
         </is>
       </c>
-      <c r="G9" s="21" t="inlineStr">
+      <c r="G9" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1282,27 +1323,27 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>訓後晚餐</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>150 g（半盒）</t>
         </is>
       </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>160 g</t>
         </is>
       </c>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="E10" s="23" t="inlineStr">
         <is>
           <t>約 1/2 杯</t>
         </is>
@@ -1312,7 +1353,7 @@
           <t>全蛋 2 顆</t>
         </is>
       </c>
-      <c r="G10" s="21" t="inlineStr">
+      <c r="G10" s="23" t="inlineStr">
         <is>
           <t>200 g</t>
         </is>
@@ -1324,27 +1365,27 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>睡前</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>視需要補蛋白</t>
         </is>
       </c>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="21" t="inlineStr">
+      <c r="E11" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1354,7 +1395,7 @@
           <t>乳清 0.5–1 scoop</t>
         </is>
       </c>
-      <c r="G11" s="21" t="inlineStr">
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1449,27 +1490,27 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>午餐</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>150 g（半盒）</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="23" t="inlineStr">
         <is>
           <t>200 g</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E17" s="23" t="inlineStr">
         <is>
           <t>約 0.60 杯</t>
         </is>
@@ -1479,7 +1520,7 @@
           <t>鯖魚日加台糖水煮鯖魚 1/2 罐</t>
         </is>
       </c>
-      <c r="G17" s="21" t="inlineStr">
+      <c r="G17" s="23" t="inlineStr">
         <is>
           <t>300 g</t>
         </is>
@@ -1491,27 +1532,27 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>下午茶</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="C18" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="23" t="inlineStr">
         <is>
           <t>100 g</t>
         </is>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="E18" s="23" t="inlineStr">
         <is>
           <t>約 0.30 杯</t>
         </is>
@@ -1521,7 +1562,7 @@
           <t>全蛋 2 顆＋乳清 1–1.5 scoop</t>
         </is>
       </c>
-      <c r="G18" s="21" t="inlineStr">
+      <c r="G18" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1533,27 +1574,27 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>晚餐</t>
         </is>
       </c>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>150 g（半盒）</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="23" t="inlineStr">
         <is>
           <t>150 g</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E19" s="23" t="inlineStr">
         <is>
           <t>約 0.45 杯</t>
         </is>
@@ -1563,7 +1604,7 @@
           <t>全蛋 2 顆</t>
         </is>
       </c>
-      <c r="G19" s="21" t="inlineStr">
+      <c r="G19" s="23" t="inlineStr">
         <is>
           <t>300 g</t>
         </is>
@@ -1644,27 +1685,27 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t>週一</t>
         </is>
       </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B26" s="23" t="inlineStr">
         <is>
           <t>訓練日</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C26" s="23" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D26" s="21" t="inlineStr">
+      <c r="D26" s="23" t="inlineStr">
         <is>
           <t>約2杯</t>
         </is>
       </c>
-      <c r="E26" s="21" t="inlineStr">
+      <c r="E26" s="23" t="inlineStr">
         <is>
           <t>1/2罐</t>
         </is>
@@ -1676,27 +1717,27 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>週二</t>
         </is>
       </c>
-      <c r="B27" s="21" t="inlineStr">
+      <c r="B27" s="23" t="inlineStr">
         <is>
           <t>訓練日</t>
         </is>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C27" s="23" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D27" s="23" t="inlineStr">
         <is>
           <t>約2杯</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E27" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1708,27 +1749,27 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>週三</t>
         </is>
       </c>
-      <c r="B28" s="21" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>休息日</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr">
+      <c r="C28" s="23" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D28" s="21" t="inlineStr">
+      <c r="D28" s="23" t="inlineStr">
         <is>
           <t>約1.4杯</t>
         </is>
       </c>
-      <c r="E28" s="21" t="inlineStr">
+      <c r="E28" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1740,27 +1781,27 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>週四</t>
         </is>
       </c>
-      <c r="B29" s="21" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>訓練日</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C29" s="23" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="23" t="inlineStr">
         <is>
           <t>約2杯</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="E29" s="23" t="inlineStr">
         <is>
           <t>1/2罐</t>
         </is>
@@ -1772,27 +1813,27 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>週五</t>
         </is>
       </c>
-      <c r="B30" s="21" t="inlineStr">
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t>休息日</t>
         </is>
       </c>
-      <c r="C30" s="21" t="inlineStr">
+      <c r="C30" s="23" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D30" s="21" t="inlineStr">
+      <c r="D30" s="23" t="inlineStr">
         <is>
           <t>約1.4杯</t>
         </is>
       </c>
-      <c r="E30" s="21" t="inlineStr">
+      <c r="E30" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1804,27 +1845,27 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>週六</t>
         </is>
       </c>
-      <c r="B31" s="21" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>訓練日</t>
         </is>
       </c>
-      <c r="C31" s="21" t="inlineStr">
+      <c r="C31" s="23" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D31" s="21" t="inlineStr">
+      <c r="D31" s="23" t="inlineStr">
         <is>
           <t>約2杯</t>
         </is>
       </c>
-      <c r="E31" s="21" t="inlineStr">
+      <c r="E31" s="23" t="inlineStr">
         <is>
           <t>1/2罐</t>
         </is>
@@ -1836,27 +1877,27 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="21" t="inlineStr">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>週日</t>
         </is>
       </c>
-      <c r="B32" s="21" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>休息日</t>
         </is>
       </c>
-      <c r="C32" s="21" t="inlineStr">
+      <c r="C32" s="23" t="inlineStr">
         <is>
           <t>1盒</t>
         </is>
       </c>
-      <c r="D32" s="21" t="inlineStr">
+      <c r="D32" s="23" t="inlineStr">
         <is>
           <t>約1.4杯</t>
         </is>
       </c>
-      <c r="E32" s="21" t="inlineStr">
+      <c r="E32" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1887,84 +1928,84 @@
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="21" t="inlineStr">
+      <c r="A37" s="23" t="inlineStr">
         <is>
           <t>雞胸 300 g/盒</t>
         </is>
       </c>
-      <c r="B37" s="21" t="inlineStr">
+      <c r="B37" s="23" t="inlineStr">
         <is>
           <t>7 盒</t>
         </is>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>台糖水煮鯖魚</t>
         </is>
       </c>
-      <c r="B38" s="21" t="inlineStr">
+      <c r="B38" s="23" t="inlineStr">
         <is>
           <t>2 罐即可（實吃 1.5 罐）</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>雞蛋</t>
         </is>
       </c>
-      <c r="B39" s="21" t="inlineStr">
+      <c r="B39" s="23" t="inlineStr">
         <is>
           <t>28 顆</t>
         </is>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>生米</t>
         </is>
       </c>
-      <c r="B40" s="21" t="inlineStr">
+      <c r="B40" s="23" t="inlineStr">
         <is>
           <t>約 12.2 米杯/週</t>
         </is>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="21" t="inlineStr">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>香蕉</t>
         </is>
       </c>
-      <c r="B41" s="21" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>至少 4 根</t>
         </is>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="21" t="inlineStr">
+      <c r="A42" s="23" t="inlineStr">
         <is>
           <t>青菜</t>
         </is>
       </c>
-      <c r="B42" s="21" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>約 3.4 kg/週以上</t>
         </is>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="23" t="inlineStr">
         <is>
           <t>乳清</t>
         </is>
       </c>
-      <c r="B43" s="21" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>約 11–14 scoop/週</t>
         </is>

</xml_diff>

<commit_message>
Update protein product and today log
</commit_message>
<xml_diff>
--- a/data/減脂追蹤.xlsx
+++ b/data/減脂追蹤.xlsx
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>365</v>
+        <v>415.2</v>
       </c>
       <c r="D5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$12,IF($B5="REST",'設定'!$D$12,"")))</f>
@@ -719,7 +719,7 @@
         <v/>
       </c>
       <c r="F5" s="6" t="n">
-        <v>38</v>
+        <v>35.2</v>
       </c>
       <c r="G5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$13,IF($B5="REST",'設定'!$D$13,"")))</f>
@@ -730,7 +730,7 @@
         <v/>
       </c>
       <c r="I5" s="6" t="n">
-        <v>31</v>
+        <v>38.8</v>
       </c>
       <c r="J5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$14,IF($B5="REST",'設定'!$D$14,"")))</f>
@@ -741,7 +741,7 @@
         <v/>
       </c>
       <c r="L5" s="6" t="n">
-        <v>12</v>
+        <v>14.2</v>
       </c>
       <c r="M5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$15,IF($B5="REST",'設定'!$D$15,"")))</f>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>乳清 1 scoop＋香蕉 1 根</t>
+          <t>樂維根麵茶植物蛋白 1 份（40 g）＋香蕉 1 根</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>乳清 0.5–1 scoop</t>
+          <t>樂維根麵茶植物蛋白 0.5–1 份</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>全蛋 4 顆＋乳清 1.5–2 scoop＋香蕉 1 根</t>
+          <t>全蛋 4 顆＋樂維根麵茶植物蛋白 1.5–2 份＋香蕉 1 根</t>
         </is>
       </c>
       <c r="G12" s="22" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>全蛋 2 顆＋乳清 1–1.5 scoop</t>
+          <t>全蛋 2 顆＋樂維根麵茶植物蛋白 1–1.5 份</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>把原早餐內容移到下午茶；若蛋白質不足再補 0.5 scoop</t>
+          <t>把原早餐內容移到下午茶；若蛋白質不足再補 0.5 份</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>全蛋 4 顆＋乳清 1–1.5 scoop</t>
+          <t>全蛋 4 顆＋樂維根麵茶植物蛋白 1–1.5 份</t>
         </is>
       </c>
       <c r="G20" s="22" t="inlineStr">
@@ -2002,12 +2002,12 @@
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>乳清</t>
+          <t>樂維根麵茶植物蛋白</t>
         </is>
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>約 11–14 scoop/週</t>
+          <t>約 11–14 份/週</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>可放午餐或下午茶；蛋白質不足時再補乳清或無糖豆漿</t>
+          <t>可放午餐或下午茶；蛋白質不足時再補樂維根麵茶植物蛋白或無糖豆漿</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Update today macro log
</commit_message>
<xml_diff>
--- a/data/減脂追蹤.xlsx
+++ b/data/減脂追蹤.xlsx
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>415.2</v>
+        <v>985.4</v>
       </c>
       <c r="D5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$12,IF($B5="REST",'設定'!$D$12,"")))</f>
@@ -719,7 +719,7 @@
         <v/>
       </c>
       <c r="F5" s="6" t="n">
-        <v>35.2</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="G5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$13,IF($B5="REST",'設定'!$D$13,"")))</f>
@@ -730,7 +730,7 @@
         <v/>
       </c>
       <c r="I5" s="6" t="n">
-        <v>38.8</v>
+        <v>106.3</v>
       </c>
       <c r="J5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$14,IF($B5="REST",'設定'!$D$14,"")))</f>
@@ -741,7 +741,7 @@
         <v/>
       </c>
       <c r="L5" s="6" t="n">
-        <v>14.2</v>
+        <v>21.6</v>
       </c>
       <c r="M5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$15,IF($B5="REST",'設定'!$D$15,"")))</f>

</xml_diff>

<commit_message>
Update 2026-09-16 dinner log
</commit_message>
<xml_diff>
--- a/data/減脂追蹤.xlsx
+++ b/data/減脂追蹤.xlsx
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>985.4</v>
+        <v>1789.4</v>
       </c>
       <c r="D5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$12,IF($B5="REST",'設定'!$D$12,"")))</f>
@@ -719,7 +719,7 @@
         <v/>
       </c>
       <c r="F5" s="6" t="n">
-        <v>92.09999999999999</v>
+        <v>151.7</v>
       </c>
       <c r="G5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$13,IF($B5="REST",'設定'!$D$13,"")))</f>
@@ -730,7 +730,7 @@
         <v/>
       </c>
       <c r="I5" s="6" t="n">
-        <v>106.3</v>
+        <v>212.7</v>
       </c>
       <c r="J5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$14,IF($B5="REST",'設定'!$D$14,"")))</f>
@@ -741,7 +741,7 @@
         <v/>
       </c>
       <c r="L5" s="6" t="n">
-        <v>21.6</v>
+        <v>34.8</v>
       </c>
       <c r="M5" s="7">
         <f>IF($B5="","",IF($B5="TRAINING",'設定'!$B$15,IF($B5="REST",'設定'!$D$15,"")))</f>

</xml_diff>